<commit_message>
Creación superusuario + actualización excel
</commit_message>
<xml_diff>
--- a/Planificacion_Grupo03_E2.xlsx
+++ b/Planificacion_Grupo03_E2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deusto\Desktop\IW-GRUPO3-E2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D72A00F-2D61-4911-9973-570CD0276878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4047A1-2968-4061-BA0E-2D7081B569AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -463,7 +463,7 @@
     <col min="6" max="6" width="49.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,7 +503,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -536,9 +536,11 @@
       <c r="D4" s="3">
         <v>46132</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="E4" s="3">
+        <v>46132</v>
+      </c>
       <c r="F4" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Listado y detalle Proveedores
</commit_message>
<xml_diff>
--- a/Planificacion_Grupo03_E2.xlsx
+++ b/Planificacion_Grupo03_E2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deusto\Desktop\IW-GRUPO3-E2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0325D045-F5A6-4594-A7B9-C318D3B3A8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9FEA8BE-F065-4771-8A72-B6A897B35B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="19">
   <si>
     <t>Nº</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t xml:space="preserve">implementar dashboard con estadísticas, navegación centralizada y cálculo de totales en órdenes, así como prueba de botón Nuevo Artículo </t>
+  </si>
+  <si>
+    <t>Listado y detalle Proveedores</t>
   </si>
 </sst>
 </file>
@@ -518,7 +521,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -538,7 +541,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -668,12 +671,24 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="2"/>
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="3">
+        <v>46143</v>
+      </c>
+      <c r="E10" s="3">
+        <v>46143</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="H10" s="2" t="s">
         <v>12</v>
       </c>

</xml_diff>